<commit_message>
Update fi6-tasks.xlsx — replace subtitles with full task descriptions
Each Description cell now explains exactly what Logan needs to do:
read the dossier, answer 5 questions, and the 60% pass threshold.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fi6-tasks.xlsx
+++ b/fi6-tasks.xlsx
@@ -587,7 +587,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -663,7 +663,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2" ht="50" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>6FR.AL.1</t>
@@ -696,7 +696,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Français · Arts du langage</t>
+          <t>Lis le dossier sur les 7 stratégies de lecture (prédire, inférer, synthétiser, etc.) et les types de textes. Réponds à 5 questions (choix multiple + réponse courte). Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -716,7 +716,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
+    <row r="3" ht="50" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>6FR.GR.1</t>
@@ -749,7 +749,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Français · Grammaire</t>
+          <t>Lis le dossier sur l'accord sujet-verbe et l'accord des adjectifs (genre et nombre). Réponds à 5 questions pratiques. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -769,7 +769,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
+    <row r="4" ht="50" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>6FR.GR.2</t>
@@ -802,7 +802,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Français · Conjugaison</t>
+          <t>Lis le dossier sur les deux temps du passé : passé composé (action terminée) et imparfait (habitude/état). Conjugue et identifie les temps dans 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -822,7 +822,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
+    <row r="5" ht="50" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>6FR.CO.1</t>
@@ -855,7 +855,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Français · Communication orale</t>
+          <t>Lis le dossier sur la structure d'un exposé oral (introduction, développement, conclusion) et les techniques de débat. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -875,7 +875,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="50" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>6EN.RC.1</t>
@@ -908,7 +908,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>English Language Arts · Reading</t>
+          <t>Read the dossier covering 9 literary devices: simile, metaphor, personification, alliteration, onomatopoeia, hyperbole, foreshadowing, symbolism, and imagery. Answer 5 questions. Pass mark: 60%.</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
@@ -928,7 +928,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="50" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>6EN.WF.1</t>
@@ -961,7 +961,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>English Language Arts · Writing</t>
+          <t>Read the dossier on the 5-step writing process (pre-write, draft, revise, edit, publish) and paragraph structure. Answer 5 questions. Pass mark: 60%.</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr"/>
@@ -981,7 +981,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
+    <row r="8" ht="50" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>6EN.WS.1</t>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>English Language Arts · Word Study</t>
+          <t>Read the dossier on common prefixes (un-, re-, pre-, mis-), suffixes (-tion, -ful, -less), and how to use context clues. Learn denotation vs. connotation. Answer 5 questions. Pass mark: 60%.</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
           <t>6MA.N.1</t>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Mathématiques · Nombres</t>
+          <t>Lis le dossier sur la conversion entre fractions, décimaux et pourcentages, l'addition de fractions avec le PPCD, et les nombres mixtes. Résous 5 problèmes. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr"/>
@@ -1087,7 +1087,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
+    <row r="10" ht="50" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>6MA.A.1</t>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Mathématiques · Algèbre</t>
+          <t>Lis le dossier sur l'ordre des opérations (PEDMAS), les expressions algébriques et la résolution d'équations avec des opérations inverses. Résous 5 problèmes. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr"/>
@@ -1140,7 +1140,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>6MA.G.1</t>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Mathématiques · Géométrie</t>
+          <t>Lis le dossier sur les formules d'aire (rectangle, triangle, cercle), le volume d'un prisme, et les transformations (translation, réflexion, rotation). Résous 5 problèmes. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr"/>
@@ -1193,7 +1193,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
+    <row r="12" ht="50" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>6MA.SP.1</t>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>Mathématiques · Stats &amp; Proba</t>
+          <t>Lis le dossier sur les mesures de tendance centrale (moyenne, médiane, mode, étendue) et la probabilité théorique. Calcule 5 problèmes de données. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
+    <row r="13" ht="50" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>6SC.E.1</t>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>Sciences · Électricité</t>
+          <t>Lis le dossier sur les circuits en série et en parallèle, les conducteurs et les isolants, et les règles de sécurité électrique. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr"/>
@@ -1299,7 +1299,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="50" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>6SC.SS.1</t>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>Sciences · Astronomie</t>
+          <t>Lis le dossier sur les 8 planètes dans l'ordre, les planètes telluriques vs gazeuses, les phases de la Lune, et les éclipses solaires et lunaires. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr"/>
@@ -1352,7 +1352,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="50" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
           <t>6SC.AA.1</t>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>Sciences · Air et aérodynamique</t>
+          <t>Lis le dossier sur les 4 forces du vol (portance, poids, poussée, traînée) et le principe de Bernoulli. Explique comment les avions volent en répondant à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr"/>
@@ -1405,7 +1405,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
+    <row r="16" ht="50" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>6SC.AF.1</t>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>Sciences · Arbres et forêts</t>
+          <t>Lis le dossier sur la photosynthèse, la transpiration, les 3 types de forêts (boréale, tempérée, tropicale) et les effets de la déforestation. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H16" s="14" t="inlineStr"/>
@@ -1458,7 +1458,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
+    <row r="17" ht="50" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>6SH.GE.1</t>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Sciences humaines · Géographie</t>
+          <t>Lis le dossier sur les 7 régions géographiques du Canada, leurs ressources et leur population. Identifie où se trouve l'Alberta. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr"/>
@@ -1511,7 +1511,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" ht="50" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>6SH.PA.1</t>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>Sciences humaines · Histoire</t>
+          <t>Lis le dossier sur les Premières Nations, les Métis et les Inuits, les traités, les pensionnats indiens et la réconciliation. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H18" s="17" t="inlineStr"/>
@@ -1564,7 +1564,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" ht="50" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
           <t>6SH.CF.1</t>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Sciences humaines · Histoire canadienne</t>
+          <t>Lis le dossier sur la formation du Canada en 1867, les 4 provinces fondatrices, les raisons de la Confédération et l'adhésion de l'Alberta en 1905. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr"/>
@@ -1617,7 +1617,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
+    <row r="20" ht="50" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>6SH.GV.1</t>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Sciences humaines · Gouvernement</t>
+          <t>Lis le dossier sur les 3 paliers de gouvernement (fédéral, provincial, municipal), leurs responsabilités et le fonctionnement du Parlement. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H20" s="17" t="inlineStr"/>
@@ -1670,7 +1670,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
+    <row r="21" ht="50" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
         <is>
           <t>6HL.WB.1</t>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="G21" s="21" t="inlineStr">
         <is>
-          <t>Santé · Bien-être physique</t>
+          <t>Lis le dossier sur les systèmes digestif, circulatoire, respiratoire et musculo-squelettique, et les 4 dimensions de la santé. Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr"/>
@@ -1723,7 +1723,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
+    <row r="22" ht="50" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
           <t>6HL.LS.1</t>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="G22" s="21" t="inlineStr">
         <is>
-          <t>Santé · Compétences de vie</t>
+          <t>Lis le dossier sur le modèle de prise de décision en 5 étapes, les stratégies saines de gestion du stress et les compétences sociales (empathie, refus positif). Réponds à 5 questions. Résultat de passage : 60 %.</t>
         </is>
       </c>
       <c r="H22" s="20" t="inlineStr"/>

</xml_diff>

<commit_message>
Update fi6-tasks.xlsx with full Q&A in Description column for worksheet modal
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fi6-tasks.xlsx
+++ b/fi6-tasks.xlsx
@@ -154,13 +154,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -169,49 +169,49 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -586,10 +586,10 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
@@ -663,7 +663,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="50" customHeight="1">
+    <row r="2" ht="110" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>6FR.AL.1</t>
@@ -696,7 +696,16 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les 7 stratégies de lecture (prédire, inférer, synthétiser, etc.) et les types de textes. Réponds à 5 questions (choix multiple + réponse courte). Résultat de passage : 60 %.</t>
+          <t>Q1: Quelle stratégie consiste à "lire entre les lignes" ?
+   Answer: Inférer
+Q2: Un article de journal qui présente des faits est un texte de type…
+   Answer: Informatif
+Q3: Quelle est la dernière étape des 7 stratégies de lecture ?
+   Answer: Synthétiser
+Q4: La stratégie de ________ consiste à former des images mentales pendant la lecture.
+   Answer: Visualiser
+Q5: Un texte qui cherche à changer ton opinion est un texte ________.
+   Answer: Persuasif</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -716,7 +725,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="50" customHeight="1">
+    <row r="3" ht="110" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>6FR.GR.1</t>
@@ -749,7 +758,16 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Lis le dossier sur l'accord sujet-verbe et l'accord des adjectifs (genre et nombre). Réponds à 5 questions pratiques. Résultat de passage : 60 %.</t>
+          <t>Q1: Choisissez la bonne forme : « Les élèves ________ attentifs. »
+   Answer: sont
+Q2: Quel est le genre et le nombre de "belles fleurs" ?
+   Answer: féminin pluriel
+Q3: Le verbe s'accorde avec son sujet en personne et en ________.
+   Answer: nombre
+Q4: « Les garçons sont grand___. » Écrivez la terminaison correcte.
+   Answer: s (grands)
+Q5: Dans « Courent vite les trois chats. » Quel est le sujet ?
+   Answer: Les trois chats</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -769,7 +787,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="50" customHeight="1">
+    <row r="4" ht="110" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>6FR.GR.2</t>
@@ -802,7 +820,16 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les deux temps du passé : passé composé (action terminée) et imparfait (habitude/état). Conjugue et identifie les temps dans 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quelle phrase utilise correctement le passé composé ?
+   Answer: J'ai mangé ce matin.
+Q2: Quel auxiliaire utilise-t-on pour conjuguer "partir" au passé composé ?
+   Answer: Être
+Q3: Conjuguez "finir" au passé composé, 1re personne singulier : j'ai ________.
+   Answer: fini
+Q4: L'imparfait décrit une action ________ ou répétée dans le passé.
+   Answer: habituelle
+Q5: Choisissez l'imparfait : « Chaque hiver, je ________ au hockey. »
+   Answer: jouais</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -822,7 +849,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1">
+    <row r="5" ht="110" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>6FR.CO.1</t>
@@ -855,7 +882,16 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Lis le dossier sur la structure d'un exposé oral (introduction, développement, conclusion) et les techniques de débat. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quelle est la structure correcte d'un exposé oral ?
+   Answer: Introduction → Développement → Conclusion
+Q2: Quel mot de transition introduit un deuxième point ?
+   Answer: Ensuite
+Q3: Dans un débat, une ________ est une réponse à l'argument de l'adversaire.
+   Answer: réfutation
+Q4: L'________ commence l'exposé et capte l'attention du public.
+   Answer: introduction
+Q5: Qu'est-ce qu'une "accroche" dans un exposé ?
+   Answer: Une phrase au début pour capter l'attention</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -875,7 +911,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1">
+    <row r="6" ht="110" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>6EN.RC.1</t>
@@ -908,7 +944,16 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Read the dossier covering 9 literary devices: simile, metaphor, personification, alliteration, onomatopoeia, hyperbole, foreshadowing, symbolism, and imagery. Answer 5 questions. Pass mark: 60%.</t>
+          <t>Q1: "The detective's hands were ice." What literary device is this?
+   Answer: Metaphor
+Q2: Which sentence uses personification?
+   Answer: The stars danced across the sky.
+Q3: "Buzz, crash, thud" — what literary device do these words represent?
+   Answer: Onomatopoeia
+Q4: A ________ compares two things using "like" or "as".
+   Answer: simile
+Q5: When a clue in a story hints at future events, this is called ________.
+   Answer: foreshadowing</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
@@ -928,7 +973,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1">
+    <row r="7" ht="110" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>6EN.WF.1</t>
@@ -961,7 +1006,16 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Read the dossier on the 5-step writing process (pre-write, draft, revise, edit, publish) and paragraph structure. Answer 5 questions. Pass mark: 60%.</t>
+          <t>Q1: In which step do you fix spelling and punctuation errors?
+   Answer: Edit (Step 4)
+Q2: What is the correct order of the writing process?
+   Answer: Pre-write → Draft → Revise → Edit → Publish
+Q3: A ________ statement tells the reader the main argument of your essay.
+   Answer: thesis
+Q4: When you reorganize paragraphs and strengthen your ideas, you are doing the ________ step.
+   Answer: revise
+Q5: What belongs in the BODY of a paragraph?
+   Answer: Topic sentence and supporting details</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr"/>
@@ -981,7 +1035,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" ht="50" customHeight="1">
+    <row r="8" ht="110" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>6EN.WS.1</t>
@@ -1014,7 +1068,16 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Read the dossier on common prefixes (un-, re-, pre-, mis-), suffixes (-tion, -ful, -less), and how to use context clues. Learn denotation vs. connotation. Answer 5 questions. Pass mark: 60%.</t>
+          <t>Q1: What does the prefix "mis-" mean?
+   Answer: Wrongly
+Q2: What does the suffix "-less" mean?
+   Answer: Without
+Q3: The dictionary meaning of a word is called its ________.
+   Answer: denotation
+Q4: The emotional feeling a word carries is called its ________.
+   Answer: connotation
+Q5: "The detective was astute, meaning she was very clever." What context clue type is this?
+   Answer: Definition clue</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr"/>
@@ -1034,7 +1097,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1">
+    <row r="9" ht="110" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
           <t>6MA.N.1</t>
@@ -1067,7 +1130,16 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Lis le dossier sur la conversion entre fractions, décimaux et pourcentages, l'addition de fractions avec le PPCD, et les nombres mixtes. Résous 5 problèmes. Résultat de passage : 60 %.</t>
+          <t>Q1: Convertis ¾ en décimal.
+   Answer: 0,75
+Q2: Convertis 0,75 en pourcentage.
+   Answer: 75 %
+Q3: Calcule ½ + ¼ = ?
+   Answer: 3/4
+Q4: Convertis 1½ en fraction impropre.
+   Answer: 3/2
+Q5: Trouve 25 % de 80.
+   Answer: 20</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr"/>
@@ -1087,7 +1159,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" ht="50" customHeight="1">
+    <row r="10" ht="110" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>6MA.A.1</t>
@@ -1120,7 +1192,16 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Lis le dossier sur l'ordre des opérations (PEDMAS), les expressions algébriques et la résolution d'équations avec des opérations inverses. Résous 5 problèmes. Résultat de passage : 60 %.</t>
+          <t>Q1: Calcule avec PEDMAS : 2 + 3 × 4 = ?
+   Answer: 14
+Q2: Résous pour n : 2n + 6 = 14. n = ?
+   Answer: 4
+Q3: Calcule : (5 + 3) × 2 - 4 = ?
+   Answer: 12
+Q4: Quelle est la différence entre une expression et une équation ?
+   Answer: Une équation a un signe égal (=)
+Q5: Résous pour n : 5n - 10 = 15. n = ?
+   Answer: 5</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr"/>
@@ -1140,7 +1221,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" ht="50" customHeight="1">
+    <row r="11" ht="110" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>6MA.G.1</t>
@@ -1173,7 +1254,16 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les formules d'aire (rectangle, triangle, cercle), le volume d'un prisme, et les transformations (translation, réflexion, rotation). Résous 5 problèmes. Résultat de passage : 60 %.</t>
+          <t>Q1: Calcule l'aire d'un rectangle de 7 cm × 4 cm.
+   Answer: 28 cm²
+Q2: Calcule l'aire d'un triangle : base = 10 cm, hauteur = 6 cm.
+   Answer: 30 cm²
+Q3: La formule pour l'aire d'un cercle est…
+   Answer: A = πr²
+Q4: Deux angles d'un triangle = 65° et 75°. Quel est le 3e angle ?
+   Answer: 40°
+Q5: Volume d'un prisme : 5 cm × 3 cm × 4 cm = ?
+   Answer: 60 cm³</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr"/>
@@ -1193,7 +1283,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" ht="50" customHeight="1">
+    <row r="12" ht="110" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>6MA.SP.1</t>
@@ -1226,7 +1316,16 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les mesures de tendance centrale (moyenne, médiane, mode, étendue) et la probabilité théorique. Calcule 5 problèmes de données. Résultat de passage : 60 %.</t>
+          <t>Q1: Données : 3, 5, 7, 5, 10. Quel est le mode ?
+   Answer: 5
+Q2: Données : 2, 4, 6, 8, 10. Quelle est la médiane ?
+   Answer: 6
+Q3: Données : 10, 2, 8, 4, 6. Quelle est la moyenne ?
+   Answer: 6
+Q4: Un dé à 6 faces. P(nombre pair) = ?
+   Answer: 1/2 (50 %)
+Q5: Étendue des données 15, 3, 9, 21, 7 = ?
+   Answer: 18</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr"/>
@@ -1246,7 +1345,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" ht="50" customHeight="1">
+    <row r="13" ht="110" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>6SC.E.1</t>
@@ -1279,7 +1378,16 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les circuits en série et en parallèle, les conducteurs et les isolants, et les règles de sécurité électrique. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Dans un circuit en série, que se passe-t-il si une ampoule brûle ?
+   Answer: Toutes les ampoules s'éteignent.
+Q2: Pourquoi les ampoules d'une maison sont-elles en parallèle ?
+   Answer: Chaque ampoule a son propre circuit — éteindre une n'affecte pas les autres.
+Q3: Le cuivre est un exemple de ________ électrique.
+   Answer: conducteur
+Q4: Le caoutchouc est un exemple d'________ électrique.
+   Answer: isolant
+Q5: Quelle mesure correspond au "flux d'électrons" ?
+   Answer: Courant (A — ampères)</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr"/>
@@ -1299,7 +1407,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" ht="50" customHeight="1">
+    <row r="14" ht="110" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>6SC.SS.1</t>
@@ -1332,7 +1440,16 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les 8 planètes dans l'ordre, les planètes telluriques vs gazeuses, les phases de la Lune, et les éclipses solaires et lunaires. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quelle est la 5e planète du Soleil ?
+   Answer: Jupiter
+Q2: Différence entre planète tellurique et gazeuse ?
+   Answer: Telluriques = rocheuses, petites. Gazeuses = grandes, composées de gaz.
+Q3: Lors d'une éclipse solaire, c'est la ________ qui bloque la lumière.
+   Answer: Lune
+Q4: Nomme la planète qui suit Mars dans l'ordre du Soleil.
+   Answer: Jupiter
+Q5: Combien de jours dure approximativement le cycle lunaire ?
+   Answer: 29,5 jours</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr"/>
@@ -1352,7 +1469,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" ht="50" customHeight="1">
+    <row r="15" ht="110" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
           <t>6SC.AA.1</t>
@@ -1385,7 +1502,16 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les 4 forces du vol (portance, poids, poussée, traînée) et le principe de Bernoulli. Explique comment les avions volent en répondant à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quelle force s'oppose au mouvement vers l'avant d'un avion ?
+   Answer: La traînée
+Q2: Selon Bernoulli, l'air qui se déplace plus vite exerce une pression…
+   Answer: Plus basse
+Q3: La force vers le haut créée par les ailes s'appelle la ________.
+   Answer: portance
+Q4: Pour qu'un avion monte, la portance doit être ________ que le poids.
+   Answer: plus grande
+Q5: Pourquoi les voitures de course ont-elles une forme profilée ?
+   Answer: Pour réduire la traînée et aller plus vite.</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr"/>
@@ -1405,7 +1531,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" ht="50" customHeight="1">
+    <row r="16" ht="110" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>6SC.AF.1</t>
@@ -1438,7 +1564,16 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>Lis le dossier sur la photosynthèse, la transpiration, les 3 types de forêts (boréale, tempérée, tropicale) et les effets de la déforestation. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quel pigment vert dans les feuilles capte l'énergie solaire ?
+   Answer: Chlorophylle
+Q2: Photosynthèse : eau + CO₂ + soleil → ________ + oxygène.
+   Answer: glucose
+Q3: Quel type de forêt trouve-t-on dans le nord du Canada ?
+   Answer: Forêt boréale
+Q4: La libération de vapeur d'eau par les stomates s'appelle la ________.
+   Answer: transpiration
+Q5: Comment la déforestation affecte-t-elle le cycle du carbone ?
+   Answer: Elle augmente le CO₂ et réduit l'absorption du carbone.</t>
         </is>
       </c>
       <c r="H16" s="14" t="inlineStr"/>
@@ -1458,7 +1593,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" ht="50" customHeight="1">
+    <row r="17" ht="110" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>6SH.GE.1</t>
@@ -1491,7 +1626,16 @@
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les 7 régions géographiques du Canada, leurs ressources et leur population. Identifie où se trouve l'Alberta. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Dans quelle région géographique se trouve l'Alberta ?
+   Answer: Les Plaines intérieures
+Q2: Quelle région est la plus densément peuplée du Canada ?
+   Answer: Les Basses-terres des Grands Lacs
+Q3: Combien de régions géographiques le Canada compte-t-il ?
+   Answer: 7
+Q4: Les peuples ________ vivent traditionnellement dans la région arctique.
+   Answer: Inuits
+Q5: Quelle est la principale ressource des Plaines intérieures ?
+   Answer: Pétrole/gaz et céréales</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr"/>
@@ -1511,7 +1655,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" ht="50" customHeight="1">
+    <row r="18" ht="110" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>6SH.PA.1</t>
@@ -1544,7 +1688,16 @@
       </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les Premières Nations, les Métis et les Inuits, les traités, les pensionnats indiens et la réconciliation. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quels sont les trois groupes de peuples autochtones reconnus au Canada ?
+   Answer: Premières Nations, Métis et Inuits
+Q2: Louis Riel est un leader célèbre du groupe des ________.
+   Answer: Métis
+Q3: Qu'est-ce qu'un traité ?
+   Answer: Un accord juridique entre le gouvernement et les nations autochtones sur les terres.
+Q4: Le processus de réparation des relations autochtones s'appelle la ________.
+   Answer: réconciliation
+Q5: Quelle était la conséquence principale des pensionnats indiens ?
+   Answer: Perte de langue, de culture et traumatisme intergénérationnel.</t>
         </is>
       </c>
       <c r="H18" s="17" t="inlineStr"/>
@@ -1564,7 +1717,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" ht="50" customHeight="1">
+    <row r="19" ht="110" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
           <t>6SH.CF.1</t>
@@ -1597,7 +1750,16 @@
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Lis le dossier sur la formation du Canada en 1867, les 4 provinces fondatrices, les raisons de la Confédération et l'adhésion de l'Alberta en 1905. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: En quelle année a eu lieu la Confédération canadienne ?
+   Answer: 1867
+Q2: Combien y a-t-il de provinces au Canada aujourd'hui ?
+   Answer: 10 provinces
+Q3: Quelles étaient les 4 premières provinces de la Confédération ?
+   Answer: Ontario, Québec, Nouvelle-Écosse, Nouveau-Brunswick
+Q4: Le premier ________ du Canada était John A. Macdonald.
+   Answer: Premier ministre
+Q5: En quelle année l'Alberta est-elle devenue une province ?
+   Answer: 1905</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr"/>
@@ -1617,7 +1779,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" ht="50" customHeight="1">
+    <row r="20" ht="110" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>6SH.GV.1</t>
@@ -1650,7 +1812,16 @@
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les 3 paliers de gouvernement (fédéral, provincial, municipal), leurs responsabilités et le fonctionnement du Parlement. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quel palier est responsable de l'éducation en Alberta ?
+   Answer: Provincial
+Q2: Quel palier est responsable de la collecte des ordures ?
+   Answer: Municipal
+Q3: La Chambre des communes et le Sénat sont les deux chambres du ________ fédéral.
+   Answer: Parlement
+Q4: Le chef du parti qui obtient le plus de sièges devient le ________.
+   Answer: Premier ministre
+Q5: L'immigration est la responsabilité de quel palier ?
+   Answer: Fédéral</t>
         </is>
       </c>
       <c r="H20" s="17" t="inlineStr"/>
@@ -1670,7 +1841,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" ht="50" customHeight="1">
+    <row r="21" ht="110" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
         <is>
           <t>6HL.WB.1</t>
@@ -1703,7 +1874,16 @@
       </c>
       <c r="G21" s="21" t="inlineStr">
         <is>
-          <t>Lis le dossier sur les systèmes digestif, circulatoire, respiratoire et musculo-squelettique, et les 4 dimensions de la santé. Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quel organe pompe le sang dans tout le corps ?
+   Answer: Le cœur
+Q2: Dans quel organe les nutriments sont-ils principalement absorbés ?
+   Answer: L'intestin grêle
+Q3: Les ________ transportent le sang DU cœur vers le reste du corps.
+   Answer: artères
+Q4: L'échange entre O₂ et CO₂ dans les poumons se fait dans les ________.
+   Answer: alvéoles
+Q5: Quelles sont les quatre dimensions de la santé complète ?
+   Answer: Physique, mentale, émotionnelle, sociale</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr"/>
@@ -1723,7 +1903,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" ht="50" customHeight="1">
+    <row r="22" ht="110" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
           <t>6HL.LS.1</t>
@@ -1756,7 +1936,16 @@
       </c>
       <c r="G22" s="21" t="inlineStr">
         <is>
-          <t>Lis le dossier sur le modèle de prise de décision en 5 étapes, les stratégies saines de gestion du stress et les compétences sociales (empathie, refus positif). Réponds à 5 questions. Résultat de passage : 60 %.</t>
+          <t>Q1: Quelle est la 1re étape du modèle de prise de décision ?
+   Answer: Identifier le problème
+Q2: Laquelle de ces stratégies est saine pour gérer le stress ?
+   Answer: La respiration profonde / l'exercice
+Q3: Comprendre les sentiments d'une autre personne s'appelle l'________.
+   Answer: empathie
+Q4: La dernière étape de la prise de décision consiste à ________ le résultat.
+   Answer: évaluer
+Q5: Qu'est-ce que le "refus positif" ?
+   Answer: Dire non poliment et avec respect.</t>
         </is>
       </c>
       <c r="H22" s="20" t="inlineStr"/>

</xml_diff>